<commit_message>
refactor: bootstrap->application 이름 수정. 스킬 정리. test: 테스트 데이타 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/RewardTable.xlsx
+++ b/input/Domains/Game/RewardTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F70DDE-A0C8-AC4C-8DE8-96EACACFA044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582F4213-947C-0A45-978A-E441ED58A560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1660" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39800" yWindow="-2320" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REWARD" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
   <si>
     <t>rewardNum</t>
   </si>
@@ -102,6 +102,42 @@
   <si>
     <t>reward_noads_month</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_mission_day_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_mission_day_002</t>
+  </si>
+  <si>
+    <t>reward_mission_day_003</t>
+  </si>
+  <si>
+    <t>reward_mission_day_004</t>
+  </si>
+  <si>
+    <t>reward_mission_day_005</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JEWEL_FREE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_mission_achieve_002</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_003</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_004</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_005</t>
   </si>
 </sst>
 </file>
@@ -485,10 +521,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
-    <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -617,6 +653,176 @@
       </c>
       <c r="E8">
         <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15">
+        <v>11</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17">
+        <v>13</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>